<commit_message>
Updated IND_grids_kan10 model - 2026-08-25 16:46
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D0E2E06-4772-435E-8DBB-F0478CC0DD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{75C5BC4E-D399-4E76-97AB-82BDB6CD9012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="70" r:id="rId1"/>
@@ -1261,52 +1261,52 @@
     <t>grid_node</t>
   </si>
   <si>
-    <t>p_w201845280-765_IND</t>
-  </si>
-  <si>
-    <t>p_w209826798-765_IND</t>
-  </si>
-  <si>
-    <t>p_w293597835-765_IND</t>
-  </si>
-  <si>
-    <t>p_w311118424-765_IND</t>
-  </si>
-  <si>
-    <t>p_w315823978-765_IND</t>
-  </si>
-  <si>
-    <t>p_w331275940-765_IND</t>
-  </si>
-  <si>
-    <t>p_w353914865-765_IND</t>
-  </si>
-  <si>
-    <t>p_w369866141-765_IND</t>
-  </si>
-  <si>
-    <t>p_w372701897-765_IND</t>
-  </si>
-  <si>
-    <t>p_w386153973-765_IND</t>
-  </si>
-  <si>
-    <t>p_w420797421-765_IND</t>
-  </si>
-  <si>
-    <t>p_w688672711-765_IND</t>
-  </si>
-  <si>
-    <t>p_w759521252-765_IND</t>
-  </si>
-  <si>
-    <t>p_w1143180503-765_IND</t>
-  </si>
-  <si>
-    <t>p_IN684-765_IND</t>
-  </si>
-  <si>
-    <t>p_w203673991-400_IND</t>
+    <t>p_Wardha_IND</t>
+  </si>
+  <si>
+    <t>p_Indore_IND</t>
+  </si>
+  <si>
+    <t>p_Solapur_IND</t>
+  </si>
+  <si>
+    <t>p_Fatehpur_IND</t>
+  </si>
+  <si>
+    <t>p_Kurnool_IND</t>
+  </si>
+  <si>
+    <t>p_Vadodara_IND</t>
+  </si>
+  <si>
+    <t>p_Korba_IND</t>
+  </si>
+  <si>
+    <t>p_Jaipur_IND</t>
+  </si>
+  <si>
+    <t>p_Moga_IND</t>
+  </si>
+  <si>
+    <t>p_Dharmapuri_IND</t>
+  </si>
+  <si>
+    <t>p_Sikandarabad_IND</t>
+  </si>
+  <si>
+    <t>p_Bhuj_IND</t>
+  </si>
+  <si>
+    <t>p_Medinipur_IND</t>
+  </si>
+  <si>
+    <t>p_Phalodi_IND</t>
+  </si>
+  <si>
+    <t>p_Rajahmundry_IND</t>
+  </si>
+  <si>
+    <t>p_Tezpur_IND</t>
   </si>
   <si>
     <t>rez_spv_IND_001</t>
@@ -1906,52 +1906,52 @@
     <t>region_com</t>
   </si>
   <si>
-    <t>e_w201845280-765_IND</t>
-  </si>
-  <si>
-    <t>e_w209826798-765_IND</t>
-  </si>
-  <si>
-    <t>e_w293597835-765_IND</t>
-  </si>
-  <si>
-    <t>e_w311118424-765_IND</t>
-  </si>
-  <si>
-    <t>e_w315823978-765_IND</t>
-  </si>
-  <si>
-    <t>e_w331275940-765_IND</t>
-  </si>
-  <si>
-    <t>e_w353914865-765_IND</t>
-  </si>
-  <si>
-    <t>e_w369866141-765_IND</t>
-  </si>
-  <si>
-    <t>e_w372701897-765_IND</t>
-  </si>
-  <si>
-    <t>e_w386153973-765_IND</t>
-  </si>
-  <si>
-    <t>e_w420797421-765_IND</t>
-  </si>
-  <si>
-    <t>e_w688672711-765_IND</t>
-  </si>
-  <si>
-    <t>e_w759521252-765_IND</t>
-  </si>
-  <si>
-    <t>e_w1143180503-765_IND</t>
-  </si>
-  <si>
-    <t>e_IN684-765_IND</t>
-  </si>
-  <si>
-    <t>e_w203673991-400_IND</t>
+    <t>e_Wardha_IND</t>
+  </si>
+  <si>
+    <t>e_Indore_IND</t>
+  </si>
+  <si>
+    <t>e_Solapur_IND</t>
+  </si>
+  <si>
+    <t>e_Fatehpur_IND</t>
+  </si>
+  <si>
+    <t>e_Kurnool_IND</t>
+  </si>
+  <si>
+    <t>e_Vadodara_IND</t>
+  </si>
+  <si>
+    <t>e_Korba_IND</t>
+  </si>
+  <si>
+    <t>e_Jaipur_IND</t>
+  </si>
+  <si>
+    <t>e_Moga_IND</t>
+  </si>
+  <si>
+    <t>e_Dharmapuri_IND</t>
+  </si>
+  <si>
+    <t>e_Sikandarabad_IND</t>
+  </si>
+  <si>
+    <t>e_Bhuj_IND</t>
+  </si>
+  <si>
+    <t>e_Medinipur_IND</t>
+  </si>
+  <si>
+    <t>e_Phalodi_IND</t>
+  </si>
+  <si>
+    <t>e_Rajahmundry_IND</t>
+  </si>
+  <si>
+    <t>e_Tezpur_IND</t>
   </si>
   <si>
     <t>elc_spv_IND_001</t>
@@ -2470,52 +2470,52 @@
     <t>lng</t>
   </si>
   <si>
-    <t>IND-e_w201845280-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w209826798-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w293597835-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w311118424-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w315823978-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w331275940-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w353914865-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w369866141-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w372701897-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w386153973-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w420797421-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w688672711-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w759521252-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w1143180503-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_IN684-765_IND</t>
-  </si>
-  <si>
-    <t>IND-e_w203673991-400_IND</t>
+    <t>IND-e_Wardha_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Indore_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Solapur_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Fatehpur_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Kurnool_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Vadodara_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Korba_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Jaipur_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Moga_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Dharmapuri_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Sikandarabad_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Bhuj_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Medinipur_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Phalodi_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Rajahmundry_IND</t>
+  </si>
+  <si>
+    <t>IND-e_Tezpur_IND</t>
   </si>
   <si>
     <t>IND-elc_spv_IND_001</t>
@@ -24146,7 +24146,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2460BD41-8D6A-42DA-A395-6E0C64C58F9F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{297D6476-3BE3-49C5-852E-DD39B93F3778}">
   <dimension ref="B9:H195"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -27884,7 +27884,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85FEAD32-5DA3-4689-9FF8-816481476390}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6138FA05-A206-425B-A6DD-FC1A4B33E2EA}">
   <dimension ref="B9:L195"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated IND_grids_kan10 model - 2026-08-31 17:09
</commit_message>
<xml_diff>
--- a/VerveStacks_IND_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_IND_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VEDA\Veda\Veda_models\vervestacks_models\VerveStacks_IND_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A92A4CD-0F62-42E1-B012-D424330BA4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369A4AC9-8133-4000-9FE5-3CC8371F2DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3966,7 +3966,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF0B5AD-A1E1-42EB-9531-825A30E3DAC7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B56A19-E4A2-493B-A5F4-5C588B6D60BA}">
   <dimension ref="B9:L195"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -31546,7 +31546,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA13FD73-828D-42F1-96CE-963352AE5D63}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAB5B0B3-985E-4A14-8D1D-1181F50E63DC}">
   <dimension ref="B9:H195"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>